<commit_message>
Add attrition, fix stage graphs
</commit_message>
<xml_diff>
--- a/results/intensive_baseline_weighted/original/log_intensive_baseline_weighted_both_1000perm.xlsx
+++ b/results/intensive_baseline_weighted/original/log_intensive_baseline_weighted_both_1000perm.xlsx
@@ -351,59 +351,147 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ver</t>
+          <t>total_shares</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>total_comments</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>total_reactions</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>verifiability</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>non_ver</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>fake</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>n_posts</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>eng</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>n_posts_covid</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>pos_b_covid</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>neutral_b_covid</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>neg_b_covid</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>n_posts_vax</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>pos_b_vax</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>neutral_b_vax</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>neg_b_vax</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2">
+        <v>-0.2453059581781583</v>
+      </c>
+      <c r="B2">
+        <v>-0.1438537241849717</v>
+      </c>
+      <c r="C2">
+        <v>-0.2261785878259515</v>
+      </c>
+      <c r="D2">
         <v>-0.05902369187389807</v>
       </c>
-      <c r="B2">
+      <c r="E2">
         <v>-0.1180894220364587</v>
       </c>
-      <c r="C2">
+      <c r="F2">
         <v>-0.04418594564373697</v>
       </c>
-      <c r="D2">
+      <c r="G2">
         <v>-0.0391402379108838</v>
       </c>
-      <c r="E2">
+      <c r="H2">
         <v>-0.1097876612486117</v>
       </c>
-      <c r="F2">
+      <c r="I2">
         <v>-0.1236533343389038</v>
+      </c>
+      <c r="J2">
+        <v>-0.005257007538364201</v>
+      </c>
+      <c r="K2">
+        <v>-0.001285393564562703</v>
+      </c>
+      <c r="L2">
+        <v>-0.000548150654991948</v>
+      </c>
+      <c r="M2">
+        <v>-0.002153009287691985</v>
+      </c>
+      <c r="N2">
+        <v>0.0006669766057435591</v>
+      </c>
+      <c r="O2">
+        <v>-0.0001903658021479122</v>
+      </c>
+      <c r="P2">
+        <v>0.0003980454816920304</v>
+      </c>
+      <c r="Q2">
+        <v>0.001174574428564644</v>
       </c>
     </row>
   </sheetData>

</xml_diff>